<commit_message>
update plots and tables output
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/Output_yearly_costs_Raw.xlsx
+++ b/CPRD Raw Analysis/Results/Output_yearly_costs_Raw.xlsx
@@ -402,25 +402,25 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>510.67</v>
+        <v>643.72</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>3650.26</v>
+        <v>9656.440000000001</v>
       </c>
       <c r="E2">
-        <v>479.4</v>
+        <v>543.55</v>
       </c>
       <c r="F2">
-        <v>370.78</v>
+        <v>504</v>
       </c>
       <c r="G2">
-        <v>168</v>
+        <v>282.69</v>
       </c>
       <c r="H2">
-        <v>692.35</v>
+        <v>840</v>
       </c>
     </row>
     <row r="3">
@@ -428,25 +428,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>593.58</v>
+        <v>276.39</v>
       </c>
       <c r="C3">
         <v>3</v>
       </c>
       <c r="D3">
-        <v>7049.25</v>
+        <v>3101.25</v>
       </c>
       <c r="E3">
-        <v>478.21</v>
+        <v>250.52</v>
       </c>
       <c r="F3">
-        <v>474.62</v>
+        <v>210</v>
       </c>
       <c r="G3">
-        <v>273</v>
+        <v>105</v>
       </c>
       <c r="H3">
-        <v>775.2</v>
+        <v>363.08</v>
       </c>
     </row>
   </sheetData>
@@ -506,25 +506,25 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>480.35</v>
+        <v>628.75</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>3650.26</v>
+        <v>9656.440000000001</v>
       </c>
       <c r="E2">
-        <v>480.36</v>
+        <v>545.88</v>
       </c>
       <c r="F2">
-        <v>336</v>
+        <v>504</v>
       </c>
       <c r="G2">
-        <v>126</v>
+        <v>252</v>
       </c>
       <c r="H2">
-        <v>672</v>
+        <v>840</v>
       </c>
     </row>
     <row r="3">
@@ -532,25 +532,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>589.03</v>
+        <v>268.04</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>7049.25</v>
+        <v>3101.25</v>
       </c>
       <c r="E3">
-        <v>479.18</v>
+        <v>251.2</v>
       </c>
       <c r="F3">
-        <v>471.6</v>
+        <v>206.39</v>
       </c>
       <c r="G3">
-        <v>273</v>
+        <v>105</v>
       </c>
       <c r="H3">
-        <v>769.37</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>